<commit_message>
Publish cache-busted workbook visual v2
</commit_message>
<xml_diff>
--- a/10-financiero/evaluacion-economica-pizzeria.xlsx
+++ b/10-financiero/evaluacion-economica-pizzeria.xlsx
@@ -32,7 +32,7 @@
     <t xml:space="preserve">EVALUACIÓN ECONÓMICA — PIZZERÍA B2B</t>
   </si>
   <si>
-    <t xml:space="preserve">Flujo libre del proyecto sin deuda · pesos nominales · horizonte de cinco años</t>
+    <t xml:space="preserve">VERSIÓN VISUAL 2 · Flujo libre sin deuda · pesos nominales · horizonte de cinco años</t>
   </si>
   <si>
     <t xml:space="preserve">Decisión del escenario activo</t>
@@ -92,7 +92,7 @@
     <t xml:space="preserve">• El flujo es económico y no incorpora deuda, intereses ni dividendos.</t>
   </si>
   <si>
-    <t xml:space="preserve">INPUTS DEL MODELO</t>
+    <t xml:space="preserve">INPUTS DEL MODELO · VERSIÓN VISUAL 2</t>
   </si>
   <si>
     <t xml:space="preserve">Edite solamente las celdas amarillas de la columna C. Todas las demás hojas usan fórmulas.</t>

</xml_diff>